<commit_message>
Update enrolment to total student strength (UG+PG+PhD) for rows 6-15
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kr4v27zxsvJFB83uytQYdr
</commit_message>
<xml_diff>
--- a/university-data/India_HE_FB_19_feed_rows6-15.xlsx
+++ b/university-data/India_HE_FB_19_feed_rows6-15.xlsx
@@ -125,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -170,6 +170,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="2" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -286,7 +287,7 @@
     <comment ref="O6" authorId="0" shapeId="0">
       <text>
         <t>Source: https://iuraipur.edu.in/assets/pdf/Engineering-2026.pdf
-NIRF 2026 data (Engineering category, IR-E-U-0635), 'Total Actual Student Strength': UG 4-yr = 168 (123 M + 45 F). Only UG row; no PG-integrated. HIGHLIGHTED: Engineering-category document only - university has no Overall/University NIRF document, so this covers B.Tech students only.</t>
+NIRF 2026 data (Engineering category, ICFAI UNIVERSITY [IR-E-U-0635]). Total Actual Student Strength: UG 4-yr 168 (only row). Ph.D pursuing (till 2024-25): Full Time 2 + Part Time 8. MD/MS 0. TOTAL = 168 + 2 + 8 = 178. HIGHLIGHTED: Engineering-only document (no Overall/University NIRF document exists) - covers B.Tech + engineering PhD only. For reference, official Annual Report 2024-25 gives whole-university Student Strength 908: https://iuraipur.edu.in/IU-Raipur-Annual-Report.pdf</t>
       </text>
     </comment>
     <comment ref="E7" authorId="0" shapeId="0">
@@ -317,6 +318,12 @@
       <text>
         <t>Source: https://iunagaland.edu.in/programs/ugprograms/bcom-major-hons
 AY 2026-27. Nagaland-domicile semester fee Rs 15,000 x 2 = Rs 30,000/year (shown in the page's 'Semester Fee' column of the scholarship table; non-domicile Rs 17,000/sem). Excludes one-time admission fee &amp; caution deposit.</t>
+      </text>
+    </comment>
+    <comment ref="S7" authorId="0" shapeId="0">
+      <text>
+        <t>Source: https://www.iunagaland.edu.in/IU-Nagaland-Annual-Report.pdf
+Official Annual Report 2024-25 (period 1 Apr 2024 - 31 Mar 2025), section 7 'Students on Roll (April 2024 - March 2025)': UG Grand Total 461 + PhD and PG Grand Total 219 (incl. 8 PhD) = 680. No NIRF data document exists for this university. HIGHLIGHTED: table follows the financial year and includes batches marked 'Outgoing (June 2024)' (UG 2021-24: 109, PG 2022-24: 65); students actually enrolled in AY 2024-25 = 680 - 109 - 65 = 506.</t>
       </text>
     </comment>
     <comment ref="E8" authorId="0" shapeId="0">
@@ -357,7 +364,7 @@
     <comment ref="O8" authorId="0" shapeId="0">
       <text>
         <t>Source: https://www.iftmuniversity.ac.in/iftmuniversity/downloads/NIRF_OVERALL_IFTMU_2026.pdf
-NIRF 2026 Overall data (IR-O-U-0515), 'Total Actual Student Strength': UG 3-yr 4745 + UG 4-yr 3601 + UG 5-yr 463 = 8809. PG (15 + 1925) and PhD excluded; no PG-integrated row.</t>
+NIRF 2026 Overall data (IFTM University [IR-O-U-0515]). Total Actual Student Strength: UG 3-yr 4745 + UG 4-yr 3601 + UG 5-yr 463 + PG 1-yr 15 + PG 2-yr 1925 = 10749. Ph.D pursuing (till 2024-25): Full Time 12 + Part Time 640. MD/MS/DNB 0. TOTAL = 10749 + 12 + 640 = 11401.</t>
       </text>
     </comment>
     <comment ref="E9" authorId="0" shapeId="0">
@@ -386,7 +393,7 @@
     <comment ref="O9" authorId="0" shapeId="0">
       <text>
         <t>Source: https://iihmr.edu.in/uploads/NIRF-IIHMR-University.pdf
-NIRF 2026 data (Management category, IR-M-U-0851). Only student-strength row is PG 2-yr (454). No UG / PG-integrated rows -&gt; UG enrolment 0 (postgraduate-only university). HIGHLIGHTED: subject-category (Management) document.</t>
+NIRF 2026 data (Management category, IIHMR University [IR-M-U-0851]). Total Actual Student Strength: PG 2-yr 454 (126 M + 328 F; only row). Ph.D pursuing (till 2024-25): Full Time 1 + Part Time 65. TOTAL = 454 + 1 + 65 = 520. HIGHLIGHTED: Management-category document (university is PG-only, so it likely covers all students).</t>
       </text>
     </comment>
     <comment ref="E10" authorId="0" shapeId="0">
@@ -421,7 +428,7 @@
     <comment ref="P10" authorId="0" shapeId="0">
       <text>
         <t>Source: https://iilm.edu/gurugram/wp-content/uploads/sites/2/2026/03/IILM-University20250128-Over-ALL.pdf
-NIRF 2025 Overall data (IR-O-S-14517), 'Total Actual Student Strength': UG 3-yr 441 + UG 4-yr 124 + UG 5-yr 195 = 760. PG (34 + 509) and PhD excluded; no PG-integrated row.</t>
+NIRF 2025 Overall data (IILM University [IR-O-S-14517], Gurugram). Total Actual Student Strength: UG 3-yr 441 + UG 4-yr 124 + UG 5-yr 195 + PG 1-yr 34 + PG 2-yr 509 = 1303. Ph.D pursuing (till 2023-24): Full Time 42 + Part Time 5. MD/MS 0. TOTAL = 1303 + 42 + 5 = 1350. (No NIRF 2026 Overall document; the 2026 Management-only document gives 317.)</t>
       </text>
     </comment>
     <comment ref="E11" authorId="0" shapeId="0">
@@ -453,10 +460,10 @@
 'Programme Fees 2026', Greater Noida section: B.Tech CSE with IBM / with Apple Rs 2,75,000 per year (4-yr 11,00,000) - most expensive B.Tech. Single annual programme fee (no separate tuition breakdown published).</t>
       </text>
     </comment>
-    <comment ref="S11" authorId="0" shapeId="0">
+    <comment ref="P11" authorId="0" shapeId="0">
       <text>
-        <t>Source: https://old.iilm.ac.in/uploads/Anual-Report-2024-25.pdf
-Annual Report 2024-25 (IILM University Greater Noida), UG students by school: 2868 + 227 + 374 + 118 + 385 = 3972 (F 1175 + M 2797). PG 685, M.Sc 8, PhD 16 excluded (grand total 4681). Used because the only NIRF document (2025 Management, IR-M-U-1219) contains PG rows only and gives no UG figure.</t>
+        <t>Source: https://iilm.edu/greater-noida/wp-content/uploads/sites/3/2026/02/final-report-submitted.pdf
+NIRF 2025-cycle data (Management category, IILM University, Greater Noida [IR-M-U-1219]; data years up to 2023-24). Total Actual Student Strength: PG 2-yr 239 (147 M + 92 F; only row). Ph.D pursuing 0 + 0. TOTAL = 239. HIGHLIGHTED: Management-only document - covers MBA students only. Whole-university figure from official Annual Report 2024-25 = 4681 (UG 3972 + PG 685 + M.Sc 8 + PhD 16): https://old.iilm.ac.in/uploads/Anual-Report-2024-25.pdf</t>
       </text>
     </comment>
     <comment ref="E12" authorId="0" shapeId="0">
@@ -491,7 +498,7 @@
     <comment ref="P12" authorId="0" shapeId="0">
       <text>
         <t>Source: https://iimtu.edu.in/uploads/images/17739221771.pdf
-NIRF 2025 Overall data (IIMT University Meerut, IR-O-C-0889), 'Total Actual Student Strength': UG 3-yr 3646 + UG 4-yr 2007 + UG 5-yr 723 = 6376. PG 2-yr 1288 and PhD excluded; no PG-integrated row.</t>
+NIRF 2025 Overall data (IIMT University Meerut [IR-O-C-0889]). Total Actual Student Strength: UG 3-yr 3646 + UG 4-yr 2007 + UG 5-yr 723 + PG 2-yr 1288 = 7664. Ph.D pursuing (till 2023-24): Full Time 303 + Part Time 79. MD/MS/DNB 0. TOTAL = 7664 + 303 + 79 = 8046.</t>
       </text>
     </comment>
     <comment ref="E13" authorId="0" shapeId="0">
@@ -527,7 +534,7 @@
     <comment ref="O13" authorId="0" shapeId="0">
       <text>
         <t>Source: https://www.iuu.ac/pdf/nirf/nirf-overall-dcs2026.pdf
-NIRF 2026 Overall data (IR-O-U-0773), 'Total Actual Student Strength': UG 3-yr 204 + UG 4-yr 523 + UG 5-yr 431 = 1158. PG (26 + 538) and PhD excluded; no PG-integrated row.</t>
+NIRF 2026 Overall data (IMS UNISON UNIVERSITY [IR-O-U-0773]). Total Actual Student Strength: UG 3-yr 204 + UG 4-yr 523 + UG 5-yr 431 + PG 1-yr 26 + PG 2-yr 538 = 1722. Ph.D pursuing (till 2024-25): Full Time 1 + Part Time 4. MD/MS/DNB 0. TOTAL = 1722 + 1 + 4 = 1727.</t>
       </text>
     </comment>
     <comment ref="E14" authorId="0" shapeId="0">
@@ -566,10 +573,10 @@
 Not listed in any NIRF 2025 subject ranking (third-party 'Management 101-125' refers to NIRF 2023).</t>
       </text>
     </comment>
-    <comment ref="P15" authorId="0" shapeId="0">
+    <comment ref="O15" authorId="0" shapeId="0">
       <text>
-        <t>Source: https://iiphg.edu.in/images/pdfs/NIRF/Submitted_Overall%20Discipline%20Report%202025.pdf
-NIRF 2025 Overall data (IR-O-U-0963). Only student-strength row is PG 2-yr (308). No UG / PG-integrated rows -&gt; UG enrolment 0 (UG programmes start only in 2026-27).</t>
+        <t>Source: https://iiphg.edu.in/images/pdfs/NIRF/Submitted%20Overall%20Discipline%20Report%202026.pdf
+NIRF 2026 Overall data (INDIAN INSTITUTE OF PUBLIC HEALTH GANDHINAGAR [IR-O-U-0963]). Total Actual Student Strength: PG 2-yr 126 (35 M + 91 F; only row). Ph.D pursuing (till 2024-25): Full Time 18 + Part Time 14. MD/MS/DNB 0. TOTAL = 126 + 18 + 14 = 158. Note: NIRF 2025 document reported PG 2-yr 308 (total 340): https://iiphg.edu.in/images/pdfs/NIRF/Submitted_Overall%20Discipline%20Report%202025.pdf</t>
       </text>
     </comment>
   </commentList>
@@ -1130,7 +1137,7 @@
       <c r="M6" s="3" t="n"/>
       <c r="N6" s="2" t="n"/>
       <c r="O6" s="21" t="n">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="P6" s="4" t="n"/>
       <c r="Q6" s="2" t="n"/>
@@ -1195,7 +1202,9 @@
       <c r="P7" s="4" t="n"/>
       <c r="Q7" s="2" t="n"/>
       <c r="R7" s="3" t="n"/>
-      <c r="S7" s="4" t="n"/>
+      <c r="S7" s="22" t="n">
+        <v>680</v>
+      </c>
       <c r="T7" s="2" t="n"/>
       <c r="U7" s="3" t="n"/>
       <c r="V7" s="4" t="n"/>
@@ -1253,8 +1262,8 @@
       <c r="L8" s="3" t="n"/>
       <c r="M8" s="3" t="n"/>
       <c r="N8" s="2" t="n"/>
-      <c r="O8" s="22" t="n">
-        <v>8809</v>
+      <c r="O8" s="23" t="n">
+        <v>11401</v>
       </c>
       <c r="P8" s="4" t="n"/>
       <c r="Q8" s="2" t="n"/>
@@ -1314,7 +1323,7 @@
       <c r="M9" s="3" t="n"/>
       <c r="N9" s="2" t="n"/>
       <c r="O9" s="21" t="n">
-        <v>0</v>
+        <v>520</v>
       </c>
       <c r="P9" s="4" t="n"/>
       <c r="Q9" s="2" t="n"/>
@@ -1376,8 +1385,8 @@
       <c r="M10" s="3" t="n"/>
       <c r="N10" s="2" t="n"/>
       <c r="O10" s="3" t="n"/>
-      <c r="P10" s="23" t="n">
-        <v>760</v>
+      <c r="P10" s="24" t="n">
+        <v>1350</v>
       </c>
       <c r="Q10" s="2" t="n"/>
       <c r="R10" s="3" t="n"/>
@@ -1438,12 +1447,12 @@
       <c r="M11" s="3" t="n"/>
       <c r="N11" s="2" t="n"/>
       <c r="O11" s="3" t="n"/>
-      <c r="P11" s="4" t="n"/>
+      <c r="P11" s="22" t="n">
+        <v>239</v>
+      </c>
       <c r="Q11" s="2" t="n"/>
       <c r="R11" s="3" t="n"/>
-      <c r="S11" s="23" t="n">
-        <v>3972</v>
-      </c>
+      <c r="S11" s="4" t="n"/>
       <c r="T11" s="2" t="n"/>
       <c r="U11" s="3" t="n"/>
       <c r="V11" s="4" t="n"/>
@@ -1500,8 +1509,8 @@
       <c r="M12" s="3" t="n"/>
       <c r="N12" s="2" t="n"/>
       <c r="O12" s="3" t="n"/>
-      <c r="P12" s="23" t="n">
-        <v>6376</v>
+      <c r="P12" s="24" t="n">
+        <v>8046</v>
       </c>
       <c r="Q12" s="2" t="n"/>
       <c r="R12" s="3" t="n"/>
@@ -1561,8 +1570,8 @@
       <c r="L13" s="3" t="n"/>
       <c r="M13" s="3" t="n"/>
       <c r="N13" s="2" t="n"/>
-      <c r="O13" s="22" t="n">
-        <v>1158</v>
+      <c r="O13" s="23" t="n">
+        <v>1727</v>
       </c>
       <c r="P13" s="4" t="n"/>
       <c r="Q13" s="2" t="n"/>
@@ -1671,10 +1680,10 @@
       <c r="L15" s="3" t="n"/>
       <c r="M15" s="3" t="n"/>
       <c r="N15" s="2" t="n"/>
-      <c r="O15" s="3" t="n"/>
-      <c r="P15" s="23" t="n">
-        <v>0</v>
-      </c>
+      <c r="O15" s="23" t="n">
+        <v>158</v>
+      </c>
+      <c r="P15" s="4" t="n"/>
       <c r="Q15" s="2" t="n"/>
       <c r="R15" s="3" t="n"/>
       <c r="S15" s="4" t="n"/>

</xml_diff>